<commit_message>
feat: Update the readme and the dashboard scorer page
</commit_message>
<xml_diff>
--- a/public/data/world_cup_2026.xlsx
+++ b/public/data/world_cup_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santanub\dev\fifa_2026\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{552C0918-13CA-42E3-B493-D6C50FD173BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23DAA83D-9F10-4BC5-84C9-46FD4574C5E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Matches" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="131">
   <si>
     <t>MatchID</t>
   </si>
@@ -29,6 +29,18 @@
     <t>Date</t>
   </si>
   <si>
+    <t>Team 1</t>
+  </si>
+  <si>
+    <t>Team 2</t>
+  </si>
+  <si>
+    <t>Team 1 Score</t>
+  </si>
+  <si>
+    <t>Team 2 Score</t>
+  </si>
+  <si>
     <t>Stage</t>
   </si>
   <si>
@@ -38,22 +50,136 @@
     <t>Group</t>
   </si>
   <si>
+    <t>Team 1 scorers</t>
+  </si>
+  <si>
+    <t>Team 2 scorers</t>
+  </si>
+  <si>
+    <t>South Africa</t>
+  </si>
+  <si>
+    <t>Mexico</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Jullan, Raul</t>
+  </si>
+  <si>
+    <t>S Korea</t>
+  </si>
+  <si>
+    <t>Czechia</t>
+  </si>
+  <si>
+    <t>Hawang in-beom, Hyeon-gyu</t>
+  </si>
+  <si>
+    <t>Ladislav</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>Bosnia &amp; Herz</t>
+  </si>
+  <si>
+    <t>Draw</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Cyle Larin</t>
+  </si>
+  <si>
+    <t>Jovo Lukic</t>
+  </si>
+  <si>
     <t>USA</t>
   </si>
   <si>
+    <t>Paraguay</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Damian Bobadilla, Folarin, Folarin, Giovanni Reyna</t>
+  </si>
+  <si>
+    <t>Mauricio</t>
+  </si>
+  <si>
+    <t>Qatar</t>
+  </si>
+  <si>
+    <t>Switzerland</t>
+  </si>
+  <si>
     <t>TBD</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Mexico</t>
-  </si>
-  <si>
-    <t>Canada</t>
-  </si>
-  <si>
-    <t>B</t>
+    <t>Brazil</t>
+  </si>
+  <si>
+    <t>Morocco</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Haiti</t>
+  </si>
+  <si>
+    <t>Scotland</t>
+  </si>
+  <si>
+    <t>Australia</t>
+  </si>
+  <si>
+    <t>Turkey</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>Curacao</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>Netherland</t>
+  </si>
+  <si>
+    <t>Japan</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Ivory Coast</t>
+  </si>
+  <si>
+    <t>Ecuador</t>
+  </si>
+  <si>
+    <t>Sweden</t>
+  </si>
+  <si>
+    <t>Tunisia</t>
+  </si>
+  <si>
+    <t>Spain</t>
+  </si>
+  <si>
+    <t>Cabo Verde</t>
+  </si>
+  <si>
+    <t>H</t>
   </si>
   <si>
     <t>TeamName</t>
@@ -71,48 +197,6 @@
     <t>CA</t>
   </si>
   <si>
-    <t>South Africa</t>
-  </si>
-  <si>
-    <t>Team 1</t>
-  </si>
-  <si>
-    <t>Team 2</t>
-  </si>
-  <si>
-    <t>Team 1 Score</t>
-  </si>
-  <si>
-    <t>Team 2 Score</t>
-  </si>
-  <si>
-    <t>Czechia</t>
-  </si>
-  <si>
-    <t>Bosnia &amp; Herz</t>
-  </si>
-  <si>
-    <t>Paraguay</t>
-  </si>
-  <si>
-    <t>S Korea</t>
-  </si>
-  <si>
-    <t>Team 1 scorers</t>
-  </si>
-  <si>
-    <t>Team 2 scorers</t>
-  </si>
-  <si>
-    <t>Hawang in-beom, Hyeon-gyu</t>
-  </si>
-  <si>
-    <t>Ladislav</t>
-  </si>
-  <si>
-    <t>Jullan, Raul</t>
-  </si>
-  <si>
     <t>ZA</t>
   </si>
   <si>
@@ -126,6 +210,210 @@
   </si>
   <si>
     <t>PY</t>
+  </si>
+  <si>
+    <t>QA</t>
+  </si>
+  <si>
+    <t>CH</t>
+  </si>
+  <si>
+    <t>BR</t>
+  </si>
+  <si>
+    <t>MA</t>
+  </si>
+  <si>
+    <t>HT</t>
+  </si>
+  <si>
+    <t>GB-SCT</t>
+  </si>
+  <si>
+    <t>AU</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>CV</t>
+  </si>
+  <si>
+    <t>SE</t>
+  </si>
+  <si>
+    <t>TN</t>
+  </si>
+  <si>
+    <t>CI</t>
+  </si>
+  <si>
+    <t>EC</t>
+  </si>
+  <si>
+    <t>NL</t>
+  </si>
+  <si>
+    <t>JP</t>
+  </si>
+  <si>
+    <t>CW</t>
+  </si>
+  <si>
+    <t>Argentina</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>AR</t>
+  </si>
+  <si>
+    <t>England</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>GB-ENG</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>FR</t>
+  </si>
+  <si>
+    <t>Croatia</t>
+  </si>
+  <si>
+    <t>HR</t>
+  </si>
+  <si>
+    <t>Ghana</t>
+  </si>
+  <si>
+    <t>GH</t>
+  </si>
+  <si>
+    <t>Panama</t>
+  </si>
+  <si>
+    <t>PA</t>
+  </si>
+  <si>
+    <t>Colombia</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>CO</t>
+  </si>
+  <si>
+    <t>Portugal</t>
+  </si>
+  <si>
+    <t>PT</t>
+  </si>
+  <si>
+    <t>DR Congo</t>
+  </si>
+  <si>
+    <t>CD</t>
+  </si>
+  <si>
+    <t>Uzbekistan</t>
+  </si>
+  <si>
+    <t>UZ</t>
+  </si>
+  <si>
+    <t>Algeria</t>
+  </si>
+  <si>
+    <t>DZ</t>
+  </si>
+  <si>
+    <t>Austria</t>
+  </si>
+  <si>
+    <t>AT</t>
+  </si>
+  <si>
+    <t>Jordan</t>
+  </si>
+  <si>
+    <t>JO</t>
+  </si>
+  <si>
+    <t>Senegal</t>
+  </si>
+  <si>
+    <t>SN</t>
+  </si>
+  <si>
+    <t>Iraq</t>
+  </si>
+  <si>
+    <t>IQ</t>
+  </si>
+  <si>
+    <t>Norway</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>Saudi Arabia</t>
+  </si>
+  <si>
+    <t>SA</t>
+  </si>
+  <si>
+    <t>Uruguay</t>
+  </si>
+  <si>
+    <t>UY</t>
+  </si>
+  <si>
+    <t>Iran</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>IR</t>
+  </si>
+  <si>
+    <t>New Zealand</t>
+  </si>
+  <si>
+    <t>NZ</t>
+  </si>
+  <si>
+    <t>Egypt</t>
+  </si>
+  <si>
+    <t>EG</t>
+  </si>
+  <si>
+    <t>Belgium</t>
+  </si>
+  <si>
+    <t>BE</t>
+  </si>
+  <si>
+    <t>Jordon</t>
   </si>
 </sst>
 </file>
@@ -163,7 +451,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -503,11 +791,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="9.9140625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -517,45 +802,45 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2">
         <v>46185</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -564,30 +849,30 @@
         <v>2</v>
       </c>
       <c r="G2" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="K2" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3">
         <v>46185</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -596,183 +881,1015 @@
         <v>2</v>
       </c>
       <c r="G3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H3" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="I3" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="J3" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="K3" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4">
         <v>46186</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" t="s">
         <v>22</v>
       </c>
-      <c r="G4" t="s">
-        <v>4</v>
-      </c>
-      <c r="H4" t="s">
-        <v>6</v>
-      </c>
-      <c r="I4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5">
         <v>46186</v>
       </c>
       <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A6">
         <v>5</v>
       </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="B6">
+        <v>46187</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="I5" t="s">
+      <c r="B7">
+        <v>46187</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" t="s">
+        <v>8</v>
+      </c>
+      <c r="H7" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>46187</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>46187</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>46187</v>
+      </c>
+      <c r="C10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" t="s">
+        <v>8</v>
+      </c>
+      <c r="H10" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A11">
         <v>10</v>
+      </c>
+      <c r="B11">
+        <v>46188</v>
+      </c>
+      <c r="C11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>46188</v>
+      </c>
+      <c r="C12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" t="s">
+        <v>47</v>
+      </c>
+      <c r="G12" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>46188</v>
+      </c>
+      <c r="C13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" t="s">
+        <v>8</v>
+      </c>
+      <c r="H13" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>46188</v>
+      </c>
+      <c r="C14" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" t="s">
+        <v>51</v>
+      </c>
+      <c r="G14" t="s">
+        <v>8</v>
+      </c>
+      <c r="H14" t="s">
+        <v>32</v>
+      </c>
+      <c r="I14" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1">
+        <v>46189</v>
+      </c>
+      <c r="C15" t="s">
+        <v>128</v>
+      </c>
+      <c r="D15" t="s">
+        <v>126</v>
+      </c>
+      <c r="G15" t="s">
+        <v>8</v>
+      </c>
+      <c r="H15" t="s">
+        <v>32</v>
+      </c>
+      <c r="I15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1">
+        <v>46189</v>
+      </c>
+      <c r="C16" t="s">
+        <v>117</v>
+      </c>
+      <c r="D16" t="s">
+        <v>119</v>
+      </c>
+      <c r="G16" t="s">
+        <v>8</v>
+      </c>
+      <c r="H16" t="s">
+        <v>32</v>
+      </c>
+      <c r="I16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1">
+        <v>46189</v>
+      </c>
+      <c r="C17" t="s">
+        <v>121</v>
+      </c>
+      <c r="D17" t="s">
+        <v>124</v>
+      </c>
+      <c r="G17" t="s">
+        <v>8</v>
+      </c>
+      <c r="H17" t="s">
+        <v>32</v>
+      </c>
+      <c r="I17" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1">
+        <v>46190</v>
+      </c>
+      <c r="C18" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18" t="s">
+        <v>111</v>
+      </c>
+      <c r="G18" t="s">
+        <v>8</v>
+      </c>
+      <c r="H18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1">
+        <v>46190</v>
+      </c>
+      <c r="C19" t="s">
+        <v>113</v>
+      </c>
+      <c r="D19" t="s">
+        <v>115</v>
+      </c>
+      <c r="G19" t="s">
+        <v>8</v>
+      </c>
+      <c r="H19" t="s">
+        <v>32</v>
+      </c>
+      <c r="I19" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1">
+        <v>46190</v>
+      </c>
+      <c r="C20" t="s">
+        <v>81</v>
+      </c>
+      <c r="D20" t="s">
+        <v>105</v>
+      </c>
+      <c r="G20" t="s">
+        <v>8</v>
+      </c>
+      <c r="H20" t="s">
+        <v>32</v>
+      </c>
+      <c r="I20" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1">
+        <v>46190</v>
+      </c>
+      <c r="C21" t="s">
+        <v>107</v>
+      </c>
+      <c r="D21" t="s">
+        <v>130</v>
+      </c>
+      <c r="G21" t="s">
+        <v>8</v>
+      </c>
+      <c r="H21" t="s">
+        <v>32</v>
+      </c>
+      <c r="I21" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:B1 A4 A2 A3 G3 C4 G2 G1:I1 I2 I3 F4:G4 I4" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:K14" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>16</v>
       </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="B11" t="s">
         <v>22</v>
       </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="C11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>34</v>
+      </c>
+      <c r="B13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C27" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>81</v>
+      </c>
+      <c r="B28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>84</v>
+      </c>
+      <c r="B29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>87</v>
+      </c>
+      <c r="B30" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>90</v>
+      </c>
+      <c r="B31" t="s">
+        <v>85</v>
+      </c>
+      <c r="C31" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>92</v>
+      </c>
+      <c r="B32" t="s">
+        <v>85</v>
+      </c>
+      <c r="C32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>94</v>
+      </c>
+      <c r="B33" t="s">
+        <v>85</v>
+      </c>
+      <c r="C33" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>96</v>
+      </c>
+      <c r="B34" t="s">
+        <v>97</v>
+      </c>
+      <c r="C34" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>99</v>
+      </c>
+      <c r="B35" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>101</v>
+      </c>
+      <c r="B36" t="s">
+        <v>97</v>
+      </c>
+      <c r="C36" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>103</v>
+      </c>
+      <c r="B37" t="s">
+        <v>97</v>
+      </c>
+      <c r="C37" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>105</v>
+      </c>
+      <c r="B38" t="s">
+        <v>82</v>
+      </c>
+      <c r="C38" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>107</v>
+      </c>
+      <c r="B39" t="s">
+        <v>82</v>
+      </c>
+      <c r="C39" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>109</v>
+      </c>
+      <c r="B40" t="s">
+        <v>82</v>
+      </c>
+      <c r="C40" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>111</v>
+      </c>
+      <c r="B41" t="s">
+        <v>88</v>
+      </c>
+      <c r="C41" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>113</v>
+      </c>
+      <c r="B42" t="s">
+        <v>88</v>
+      </c>
+      <c r="C42" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>115</v>
+      </c>
+      <c r="B43" t="s">
+        <v>88</v>
+      </c>
+      <c r="C43" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>117</v>
+      </c>
+      <c r="B44" t="s">
+        <v>52</v>
+      </c>
+      <c r="C44" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>119</v>
+      </c>
+      <c r="B45" t="s">
+        <v>52</v>
+      </c>
+      <c r="C45" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>121</v>
+      </c>
+      <c r="B46" t="s">
+        <v>122</v>
+      </c>
+      <c r="C46" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>124</v>
+      </c>
+      <c r="B47" t="s">
+        <v>122</v>
+      </c>
+      <c r="C47" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>126</v>
+      </c>
+      <c r="B48" t="s">
+        <v>122</v>
+      </c>
+      <c r="C48" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>128</v>
+      </c>
+      <c r="B49" t="s">
+        <v>122</v>
+      </c>
+      <c r="C49" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C1 A3:C4 A2 C2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C49" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: bug fixing, footer, stat is fixed, more stat is in plan
</commit_message>
<xml_diff>
--- a/public/data/world_cup_2026.xlsx
+++ b/public/data/world_cup_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santanub\dev\fifa_2026\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23DAA83D-9F10-4BC5-84C9-46FD4574C5E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81EB5DE3-A911-48E1-B413-3E146FE5A0A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -792,9 +792,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="4" max="4" width="12.08203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -829,7 +833,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -861,7 +865,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -896,7 +900,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -931,7 +935,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -966,7 +970,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -989,7 +993,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1012,7 +1016,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1035,7 +1039,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1058,7 +1062,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1081,7 +1085,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1104,7 +1108,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1127,7 +1131,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1150,7 +1154,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1345,9 +1349,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C49"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>53</v>
       </c>
@@ -1358,7 +1362,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -1369,7 +1373,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1380,7 +1384,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -1391,7 +1395,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -1402,7 +1406,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1413,7 +1417,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1424,7 +1428,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1435,7 +1439,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -1446,7 +1450,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>30</v>
       </c>
@@ -1457,7 +1461,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>31</v>
       </c>
@@ -1468,7 +1472,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -1479,7 +1483,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -1490,7 +1494,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -1501,7 +1505,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -1512,7 +1516,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>38</v>
       </c>
@@ -1523,7 +1527,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>39</v>
       </c>
@@ -1534,7 +1538,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -1545,7 +1549,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>50</v>
       </c>
@@ -1556,7 +1560,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>51</v>
       </c>
@@ -1567,7 +1571,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -1578,7 +1582,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>49</v>
       </c>
@@ -1589,7 +1593,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>46</v>
       </c>
@@ -1600,7 +1604,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>47</v>
       </c>
@@ -1611,7 +1615,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>43</v>
       </c>
@@ -1622,7 +1626,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>44</v>
       </c>
@@ -1633,7 +1637,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>41</v>
       </c>
@@ -1644,7 +1648,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>81</v>
       </c>
@@ -1655,7 +1659,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>84</v>
       </c>
@@ -1666,7 +1670,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>87</v>
       </c>
@@ -1677,7 +1681,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>90</v>
       </c>
@@ -1688,7 +1692,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>92</v>
       </c>
@@ -1699,7 +1703,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>94</v>
       </c>
@@ -1710,7 +1714,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>96</v>
       </c>
@@ -1721,7 +1725,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>99</v>
       </c>
@@ -1732,7 +1736,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>101</v>
       </c>
@@ -1743,7 +1747,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>103</v>
       </c>
@@ -1754,7 +1758,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>105</v>
       </c>
@@ -1765,7 +1769,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>107</v>
       </c>
@@ -1776,7 +1780,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>109</v>
       </c>
@@ -1787,7 +1791,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>111</v>
       </c>
@@ -1798,7 +1802,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>113</v>
       </c>
@@ -1809,7 +1813,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>115</v>
       </c>
@@ -1820,7 +1824,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>117</v>
       </c>
@@ -1831,7 +1835,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>119</v>
       </c>
@@ -1842,7 +1846,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>121</v>
       </c>
@@ -1853,7 +1857,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>124</v>
       </c>
@@ -1864,7 +1868,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>126</v>
       </c>
@@ -1875,7 +1879,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>128</v>
       </c>

</xml_diff>

<commit_message>
Yellow and red cards stat shown
</commit_message>
<xml_diff>
--- a/public/data/world_cup_2026.xlsx
+++ b/public/data/world_cup_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santanub\dev\fifa_2026\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD44031D-7BE3-40A2-8D03-C609901CC262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E70B005-3B4D-4359-80EE-702CD2DEC24A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="141">
   <si>
     <t>MatchID</t>
   </si>
@@ -437,6 +437,18 @@
   </si>
   <si>
     <t>Team 2 Yellow</t>
+  </si>
+  <si>
+    <t>Vinicious</t>
+  </si>
+  <si>
+    <t>Ismael</t>
+  </si>
+  <si>
+    <t>John McGinn</t>
+  </si>
+  <si>
+    <t>Columbia</t>
   </si>
 </sst>
 </file>
@@ -668,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O38"/>
   <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="12.08203125" customWidth="1"/>
@@ -967,14 +979,38 @@
       <c r="D7" t="s">
         <v>35</v>
       </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
       <c r="G7" t="s">
         <v>8</v>
       </c>
       <c r="H7" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="I7" t="s">
         <v>37</v>
+      </c>
+      <c r="J7" t="s">
+        <v>137</v>
+      </c>
+      <c r="K7" t="s">
+        <v>138</v>
+      </c>
+      <c r="L7">
+        <v>2</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
@@ -990,14 +1026,35 @@
       <c r="D8" t="s">
         <v>39</v>
       </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
       <c r="G8" t="s">
         <v>8</v>
       </c>
       <c r="H8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="I8" t="s">
         <v>37</v>
+      </c>
+      <c r="K8" t="s">
+        <v>139</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
@@ -1297,6 +1354,397 @@
       </c>
       <c r="I21" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>46190</v>
+      </c>
+      <c r="C22" t="s">
+        <v>114</v>
+      </c>
+      <c r="D22" t="s">
+        <v>116</v>
+      </c>
+      <c r="G22" t="s">
+        <v>8</v>
+      </c>
+      <c r="H22" t="s">
+        <v>36</v>
+      </c>
+      <c r="I22" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1">
+        <v>46191</v>
+      </c>
+      <c r="C23" t="s">
+        <v>101</v>
+      </c>
+      <c r="D23" t="s">
+        <v>105</v>
+      </c>
+      <c r="G23" t="s">
+        <v>8</v>
+      </c>
+      <c r="H23" t="s">
+        <v>36</v>
+      </c>
+      <c r="I23" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1">
+        <v>46191</v>
+      </c>
+      <c r="C24" t="s">
+        <v>107</v>
+      </c>
+      <c r="D24" t="s">
+        <v>109</v>
+      </c>
+      <c r="G24" t="s">
+        <v>8</v>
+      </c>
+      <c r="H24" t="s">
+        <v>36</v>
+      </c>
+      <c r="I24" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1">
+        <v>46191</v>
+      </c>
+      <c r="C25" t="s">
+        <v>118</v>
+      </c>
+      <c r="D25" t="s">
+        <v>140</v>
+      </c>
+      <c r="G25" t="s">
+        <v>8</v>
+      </c>
+      <c r="H25" t="s">
+        <v>36</v>
+      </c>
+      <c r="I25" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1">
+        <v>46191</v>
+      </c>
+      <c r="C26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" t="s">
+        <v>8</v>
+      </c>
+      <c r="H26" t="s">
+        <v>36</v>
+      </c>
+      <c r="I26" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1">
+        <v>46192</v>
+      </c>
+      <c r="C27" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" t="s">
+        <v>31</v>
+      </c>
+      <c r="G27" t="s">
+        <v>8</v>
+      </c>
+      <c r="H27" t="s">
+        <v>36</v>
+      </c>
+      <c r="I27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1">
+        <v>46192</v>
+      </c>
+      <c r="C28" t="s">
+        <v>30</v>
+      </c>
+      <c r="D28" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" t="s">
+        <v>8</v>
+      </c>
+      <c r="H28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I28" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1">
+        <v>46192</v>
+      </c>
+      <c r="C29" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" t="s">
+        <v>8</v>
+      </c>
+      <c r="H29" t="s">
+        <v>36</v>
+      </c>
+      <c r="I29" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1">
+        <v>46193</v>
+      </c>
+      <c r="C30" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" t="s">
+        <v>40</v>
+      </c>
+      <c r="G30" t="s">
+        <v>8</v>
+      </c>
+      <c r="H30" t="s">
+        <v>36</v>
+      </c>
+      <c r="I30" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1">
+        <v>46193</v>
+      </c>
+      <c r="C31" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" t="s">
+        <v>35</v>
+      </c>
+      <c r="G31" t="s">
+        <v>8</v>
+      </c>
+      <c r="H31" t="s">
+        <v>36</v>
+      </c>
+      <c r="I31" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1">
+        <v>46193</v>
+      </c>
+      <c r="C32" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" t="s">
+        <v>38</v>
+      </c>
+      <c r="G32" t="s">
+        <v>8</v>
+      </c>
+      <c r="H32" t="s">
+        <v>36</v>
+      </c>
+      <c r="I32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1">
+        <v>46193</v>
+      </c>
+      <c r="C33" t="s">
+        <v>41</v>
+      </c>
+      <c r="D33" t="s">
+        <v>26</v>
+      </c>
+      <c r="G33" t="s">
+        <v>8</v>
+      </c>
+      <c r="H33" t="s">
+        <v>36</v>
+      </c>
+      <c r="I33" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1">
+        <v>46193</v>
+      </c>
+      <c r="C34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D34" t="s">
+        <v>50</v>
+      </c>
+      <c r="G34" t="s">
+        <v>8</v>
+      </c>
+      <c r="H34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I34" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1">
+        <v>46194</v>
+      </c>
+      <c r="C35" t="s">
+        <v>42</v>
+      </c>
+      <c r="D35" t="s">
+        <v>48</v>
+      </c>
+      <c r="G35" t="s">
+        <v>8</v>
+      </c>
+      <c r="H35" t="s">
+        <v>36</v>
+      </c>
+      <c r="I35" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1">
+        <v>46194</v>
+      </c>
+      <c r="C36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D36" t="s">
+        <v>43</v>
+      </c>
+      <c r="G36" t="s">
+        <v>8</v>
+      </c>
+      <c r="H36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I36" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1">
+        <v>46194</v>
+      </c>
+      <c r="C37" t="s">
+        <v>51</v>
+      </c>
+      <c r="D37" t="s">
+        <v>46</v>
+      </c>
+      <c r="G37" t="s">
+        <v>8</v>
+      </c>
+      <c r="H37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I37" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1">
+        <v>46194</v>
+      </c>
+      <c r="C38" t="s">
+        <v>52</v>
+      </c>
+      <c r="D38" t="s">
+        <v>58</v>
+      </c>
+      <c r="G38" t="s">
+        <v>8</v>
+      </c>
+      <c r="H38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I38" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>